<commit_message>
Add Novice promotion flow, skill book tabs and NPC skin tone - Add skinTone to NpcAppearance and reference the Appearance assembly - Fix NPC Idle clips pointing to an outdated animation, which sank   ShopKeeper and Blacksmith into the ground
</commit_message>
<xml_diff>
--- a/Documents/MMO_Project_Design_Data_Tracker.xlsx
+++ b/Documents/MMO_Project_Design_Data_Tracker.xlsx
@@ -1406,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="25" min="1" max="1"/>
@@ -2492,112 +2492,222 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="25" t="inlineStr">
         <is>
           <t>Combat</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="25" t="inlineStr">
         <is>
           <t>Status effect system (Stun, Poison, Silence, Blind, Freeze, Petrify)</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="25" t="inlineStr">
         <is>
           <t>StatusEffectController, wired to Fatal Blow (stun-augment) and SkillDefinition.InflictedStatus</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="25" t="inlineStr">
         <is>
           <t>Combat</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="25" t="inlineStr">
         <is>
           <t>Status effect resistance</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="25" t="inlineStr">
         <is>
           <t>See Quasi-Stats sheet</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="25" t="inlineStr">
         <is>
           <t>Character Stats</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="25" t="inlineStr">
         <is>
           <t>Monster Size/Race classification + weapon-vs-size damage table</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="25" t="inlineStr">
         <is>
           <t>WeaponSizeModifiers, real iRO Wiki Classic size table; wired on Poring (Small/Plant) and Poporing</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="25" t="inlineStr">
         <is>
           <t>Character Stats</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="25" t="inlineStr">
         <is>
           <t>Class-specific Job Level stat bonuses</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="25" t="inlineStr">
         <is>
           <t>ClassJobLevelBonusLookup, e.g. Swordman +7 STR/+2 AGI/+4 VIT/+3 DEX/+2 LUK at Job 50</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="25" t="inlineStr">
         <is>
           <t>Combat</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="25" t="inlineStr">
         <is>
           <t>Natural HP regeneration</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="25" t="inlineStr">
         <is>
           <t>PlayerHealthRegenController, boosted by Increase HP Recovery / HP Recovery While Moving passives</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="B65" s="25" t="inlineStr">
+        <is>
+          <t>Weapon own ATK added to Status ATK</t>
+        </is>
+      </c>
+      <c r="C65" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D65" s="25" t="inlineStr">
+        <is>
+          <t>ItemDefinition.weaponAttack, EquipmentManager.GetMainHandWeaponAttack; main hand only; untested in Editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="25" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="B66" s="25" t="inlineStr">
+        <is>
+          <t>Per-weapon attack speed multiplier</t>
+        </is>
+      </c>
+      <c r="C66" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D66" s="25" t="inlineStr">
+        <is>
+          <t>ItemDefinition.attackSpeedMultiplier divides the Aspd attack interval; GiantBlade 0.8, Zweihander 0.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="25" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="B67" s="25" t="inlineStr">
+        <is>
+          <t>Magnum Break HP cost and Fire after-effect</t>
+        </is>
+      </c>
+      <c r="C67" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D67" s="25" t="inlineStr">
+        <is>
+          <t>HP 20 to 16, 10 s of +20% Fire damage ignoring DEF (BuffPayload.FireDamagePercent, HealthComponent.TakePiercingDamage); untested in Editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="25" t="inlineStr">
+        <is>
+          <t>World</t>
+        </is>
+      </c>
+      <c r="B68" s="25" t="inlineStr">
+        <is>
+          <t>Point-based enemy spawn with respawn delay per monster</t>
+        </is>
+      </c>
+      <c r="C68" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D68" s="25" t="inlineStr">
+        <is>
+          <t>EnemySpawnArea: manual points, max active, 30 s default, random free point, optional boss</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="25" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="B69" s="25" t="inlineStr">
+        <is>
+          <t>Experience granted through EnemyDeathEvents</t>
+        </is>
+      </c>
+      <c r="C69" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D69" s="25" t="inlineStr">
+        <is>
+          <t>EnemyDeathHandler publishes, PlayerExperience and PlayerJobProgress subscribe; Project.AI no longer references Project.Character.Combat</t>
         </is>
       </c>
     </row>
@@ -2905,7 +3015,7 @@
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Weapon ATK bonus not yet modeled. The equipped weapon TYPE decides which stat scales damage, not the player's class — a Swordman with a bow scales off DEX too.</t>
+          <t>Status ATK is only the stat part. Final ATK = Status ATK + passive mastery bonus + the main-hand weapon's own ATK (ItemDefinition.weaponAttack, added 2026-10-10), then the buff multiplier. The equipped weapon TYPE decides which stat scales damage, not the player's class — a Swordman with a bow scales off DEX too. Staffs and books add no MATK yet.</t>
         </is>
       </c>
     </row>

</xml_diff>